<commit_message>
Formato N° Vale: AAAAMM - 00000
</commit_message>
<xml_diff>
--- a/entrada/VALES.xlsx
+++ b/entrada/VALES.xlsx
@@ -397,66 +397,87 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D5"/>
+  <cols>
+    <col min="1" max="1" width="8.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>L001</v>
+      </c>
+      <c r="B1" t="str">
         <v>Juan Pérez</v>
       </c>
-      <c r="B1">
+      <c r="C1">
         <v>1500.5</v>
       </c>
-      <c r="C1" t="str">
+      <c r="D1" t="str">
         <v>15/06/2026</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>L002</v>
+      </c>
+      <c r="B2" t="str">
         <v>María García</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>2200</v>
       </c>
-      <c r="C2" t="str">
+      <c r="D2" t="str">
         <v>20/06/2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>L003</v>
+      </c>
+      <c r="B3" t="str">
         <v>Carlos López</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>980.75</v>
       </c>
-      <c r="C3" t="str">
+      <c r="D3" t="str">
         <v>25/06/2026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>L004</v>
+      </c>
+      <c r="B4" t="str">
         <v>Ana Martínez</v>
       </c>
-      <c r="B4">
+      <c r="C4">
         <v>3100</v>
       </c>
-      <c r="C4" t="str">
+      <c r="D4" t="str">
         <v>30/06/2026</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>L005</v>
+      </c>
+      <c r="B5" t="str">
         <v>Pedro Rodríguez</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>1750.25</v>
       </c>
-      <c r="C5" t="str">
+      <c r="D5" t="str">
         <v>10/07/2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>